<commit_message>
fix(workbooks): align progress with label contract
</commit_message>
<xml_diff>
--- a/outputs/annotation_workbook/round1_annotation.xlsx
+++ b/outputs/annotation_workbook/round1_annotation.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Annotations" sheetId="1" r:id="Rab36fb13f5014cc3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="Ra04298700bff4f17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="3" r:id="R67611a8d30ef458a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Annotations" sheetId="1" r:id="Ref37861457eb494c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R32fc3d49d5d04c70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="3" r:id="R29f60eae342443f1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -318,7 +318,7 @@
   <x:dxfs count="1">
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5E9"/>
         </x:patternFill>
       </x:fill>
@@ -6722,7 +6722,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra07d5fcf204742b2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15f7f3034f0245e0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6768,10 +6768,10 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="61" t="str">
-        <x:v>Completed</x:v>
+        <x:v>Complete rows</x:v>
       </x:c>
       <x:c r="B5" s="62" t="n">
-        <x:f>B4-COUNTBLANK(Annotations!$D$2:$D$201)</x:f>
+        <x:f>COUNTIFS(Annotations!$D$2:$D$201,"&lt;&gt;",Annotations!$E$2:$E$201,"&lt;&gt;",Annotations!$F$2:$F$201,"&lt;&gt;",Annotations!$H$2:$H$201,"&lt;&gt;",Annotations!$I$2:$I$201,"&lt;&gt;",Annotations!$K$2:$K$201,"&lt;&gt;")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -7281,7 +7281,7 @@
         <x:v>Codebook version</x:v>
       </x:c>
       <x:c r="B16" s="76" t="str">
-        <x:v>1.0</x:v>
+        <x:v>1.1</x:v>
       </x:c>
       <x:c r="C16" s="76"/>
       <x:c r="D16" s="76"/>

</xml_diff>